<commit_message>
fix(export): per-subject co-panelists and Rules-screen criterion names with fractional units and lower bounds (RA-028, RA-009)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013VEQkQLJAdKCkQQkUBTXoW
</commit_message>
<xml_diff>
--- a/docs/reports/phase-12/plan-grid.xlsx
+++ b/docs/reports/phase-12/plan-grid.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="760" uniqueCount="183">
   <si>
     <t>TRƯỜNG THPT CHUYÊN</t>
   </si>
@@ -231,10 +231,10 @@
     <t>Ra đề</t>
   </si>
   <si>
-    <t>Thầy Phúc (Ra đề); Cô Quí (Phản biện); Thầy Nghĩa (Ra đề); Thầy Lộc (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Lài (Ra đề); Cô Thư (Phản biện); Thầy Nghĩa (Ra đề); Cô Lan (Phản biện)</t>
+    <t>Thầy Phúc (Ra đề); Cô Quí (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Lài (Ra đề); Cô Thư (Phản biện)</t>
   </si>
   <si>
     <t>Công nghệ</t>
@@ -243,10 +243,10 @@
     <t>Phản biện</t>
   </si>
   <si>
-    <t>Cô Lan (Ra đề); Cô Quí (Ra đề); Cô Lài (Phản biện); Thầy Nghĩa (Ra đề)</t>
-  </si>
-  <si>
-    <t>Thầy Lộc (Ra đề); Cô Quí (Ra đề); Thầy Nghĩa (Ra đề); Cô Na (Phản biện)</t>
+    <t>Thầy Nghĩa (Ra đề)</t>
+  </si>
+  <si>
+    <t>Thầy Lộc (Ra đề); Cô Quí (Ra đề)</t>
   </si>
   <si>
     <t>HIEN</t>
@@ -258,16 +258,16 @@
     <t>Phân hiệu 1 (giả lập)</t>
   </si>
   <si>
-    <t>Cô Lài (Ra đề); Thầy Phúc (Phản biện); Thầy Nghĩa (Ra đề)</t>
-  </si>
-  <si>
-    <t>Cô Tú (Ra đề); Cô Như (Phản biện); Thầy Nghĩa (Ra đề); Cô Tú (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Na (Ra đề); Cô Thư (Ra đề); Thầy Nghĩa (Ra đề); Cô Thư (Phản biện)</t>
-  </si>
-  <si>
-    <t>Thầy Phúc (Ra đề); Cô Lan (Phản biện); Thầy Nghĩa (Ra đề); Cô Quí (Phản biện)</t>
+    <t>Cô Lài (Ra đề); Thầy Phúc (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Tú (Ra đề); Cô Như (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Na (Ra đề); Cô Thư (Ra đề)</t>
+  </si>
+  <si>
+    <t>Thầy Phúc (Ra đề); Cô Lan (Phản biện)</t>
   </si>
   <si>
     <t>LAN</t>
@@ -276,16 +276,13 @@
     <t>Cô Lan</t>
   </si>
   <si>
-    <t>Cô Lài (Ra đề); Cô Bình (Ra đề); Cô Thư (Phản biện); Thầy Nghĩa (Ra đề)</t>
-  </si>
-  <si>
-    <t>Cô Quí (Ra đề); Cô Lài (Phản biện); Thầy Nghĩa (Ra đề); Cô Bình (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Lài (Ra đề); Cô Quí (Phản biện); Thầy Nghĩa (Ra đề); Thầy Phúc (Phản biện)</t>
-  </si>
-  <si>
-    <t>Thầy Phúc (Ra đề); Cô Hiền (Ra đề); Thầy Nghĩa (Ra đề); Cô Quí (Phản biện)</t>
+    <t>Cô Quí (Ra đề); Cô Lài (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Lài (Ra đề); Cô Quí (Phản biện)</t>
+  </si>
+  <si>
+    <t>Thầy Phúc (Ra đề); Cô Hiền (Ra đề)</t>
   </si>
   <si>
     <t>LAI</t>
@@ -297,19 +294,16 @@
     <t>Phân hiệu 2 (giả lập)</t>
   </si>
   <si>
-    <t>Cô Hiền (Ra đề); Thầy Phúc (Phản biện); Thầy Nghĩa (Ra đề); Cô Hiền (Phản biện)</t>
-  </si>
-  <si>
-    <t>Thầy Lộc (Ra đề); Cô Thư (Ra đề); Cô Na (Phản biện); Thầy Nghĩa (Ra đề)</t>
-  </si>
-  <si>
-    <t>Cô Bình (Ra đề); Cô Thư (Phản biện); Thầy Nghĩa (Ra đề); Cô Lan (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Lan (Ra đề); Cô Quí (Ra đề); Thầy Nghĩa (Ra đề); Cô Bình (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Lan (Ra đề); Cô Quí (Phản biện); Thầy Nghĩa (Ra đề); Thầy Phúc (Phản biện)</t>
+    <t>Cô Hiền (Ra đề); Thầy Phúc (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Bình (Ra đề); Cô Thư (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Lan (Ra đề); Cô Quí (Ra đề)</t>
+  </si>
+  <si>
+    <t>Cô Lan (Ra đề); Cô Quí (Phản biện)</t>
   </si>
   <si>
     <t>NA</t>
@@ -318,16 +312,13 @@
     <t>Cô Na</t>
   </si>
   <si>
-    <t>Thầy Lộc (Ra đề); Cô Thư (Ra đề); Thầy Nghĩa (Ra đề); Cô Lài (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Thư (Ra đề); Cô Hiền (Phản biện); Thầy Nghĩa (Ra đề); Cô Thư (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Như (Ra đề); Cô Tú (Phản biện); Thầy Nghĩa (Ra đề); Cô Quí (Phản biện)</t>
-  </si>
-  <si>
-    <t>Thầy Lộc (Ra đề); Cô Quí (Ra đề); Cô Bình (Phản biện); Thầy Nghĩa (Ra đề)</t>
+    <t>Thầy Lộc (Ra đề); Cô Thư (Ra đề)</t>
+  </si>
+  <si>
+    <t>Cô Thư (Ra đề); Cô Hiền (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Như (Ra đề); Cô Tú (Phản biện)</t>
   </si>
   <si>
     <t>NHU</t>
@@ -336,13 +327,13 @@
     <t>Cô Như</t>
   </si>
   <si>
-    <t>Cô Hiền (Ra đề); Cô Tú (Ra đề); Thầy Nghĩa (Ra đề); Cô Tú (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Tú (Ra đề); Thầy Lộc (Phản biện); Thầy Nghĩa (Ra đề)</t>
-  </si>
-  <si>
-    <t>Cô Na (Ra đề); Cô Tú (Phản biện); Thầy Nghĩa (Ra đề); Cô Quí (Phản biện)</t>
+    <t>Cô Hiền (Ra đề); Cô Tú (Ra đề)</t>
+  </si>
+  <si>
+    <t>Cô Tú (Ra đề); Thầy Lộc (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Na (Ra đề); Cô Tú (Phản biện)</t>
   </si>
   <si>
     <t>QUI</t>
@@ -354,22 +345,16 @@
     <t>Phân hiệu 4 (giả lập)</t>
   </si>
   <si>
-    <t>Cô Bình (Ra đề); Thầy Phúc (Ra đề); Thầy Nghĩa (Ra đề); Thầy Lộc (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Lan (Ra đề); Cô Lài (Phản biện); Thầy Nghĩa (Ra đề); Cô Bình (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Lan (Ra đề); Cô Lài (Ra đề); Thầy Nghĩa (Ra đề); Thầy Phúc (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Na (Ra đề); Cô Như (Ra đề); Cô Tú (Phản biện); Thầy Nghĩa (Ra đề)</t>
-  </si>
-  <si>
-    <t>Thầy Lộc (Ra đề); Cô Bình (Phản biện); Thầy Nghĩa (Ra đề); Cô Na (Phản biện)</t>
-  </si>
-  <si>
-    <t>Thầy Phúc (Ra đề); Cô Hiền (Ra đề); Cô Lan (Phản biện); Thầy Nghĩa (Ra đề)</t>
+    <t>Cô Bình (Ra đề); Thầy Phúc (Ra đề)</t>
+  </si>
+  <si>
+    <t>Cô Lan (Ra đề); Cô Lài (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Lan (Ra đề); Cô Lài (Ra đề)</t>
+  </si>
+  <si>
+    <t>Thầy Lộc (Ra đề); Cô Bình (Phản biện)</t>
   </si>
   <si>
     <t>THU</t>
@@ -378,13 +363,13 @@
     <t>Cô Thư</t>
   </si>
   <si>
-    <t>Thầy Lộc (Ra đề); Cô Na (Phản biện); Thầy Nghĩa (Ra đề); Cô Lài (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Lài (Ra đề); Cô Bình (Ra đề); Thầy Nghĩa (Ra đề); Cô Lan (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Na (Ra đề); Cô Hiền (Phản biện); Thầy Nghĩa (Ra đề)</t>
+    <t>Thầy Lộc (Ra đề); Cô Na (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Lài (Ra đề); Cô Bình (Ra đề)</t>
+  </si>
+  <si>
+    <t>Cô Na (Ra đề); Cô Hiền (Phản biện)</t>
   </si>
   <si>
     <t>TU</t>
@@ -393,13 +378,13 @@
     <t>Cô Tú</t>
   </si>
   <si>
-    <t>Cô Hiền (Ra đề); Cô Như (Phản biện); Thầy Nghĩa (Ra đề)</t>
-  </si>
-  <si>
-    <t>Cô Như (Ra đề); Thầy Lộc (Phản biện); Thầy Nghĩa (Ra đề); Cô Như (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Na (Ra đề); Cô Như (Ra đề); Thầy Nghĩa (Ra đề); Cô Quí (Phản biện)</t>
+    <t>Cô Hiền (Ra đề); Cô Như (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Như (Ra đề); Thầy Lộc (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Na (Ra đề); Cô Như (Ra đề)</t>
   </si>
   <si>
     <t>LOC</t>
@@ -408,16 +393,13 @@
     <t>Thầy Lộc</t>
   </si>
   <si>
-    <t>Cô Thư (Ra đề); Cô Na (Phản biện); Thầy Nghĩa (Ra đề); Cô Lài (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Bình (Ra đề); Thầy Phúc (Ra đề); Cô Quí (Phản biện); Thầy Nghĩa (Ra đề)</t>
-  </si>
-  <si>
-    <t>Cô Tú (Ra đề); Cô Như (Ra đề); Thầy Nghĩa (Ra đề); Cô Như (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Quí (Ra đề); Cô Bình (Phản biện); Thầy Nghĩa (Ra đề); Cô Na (Phản biện)</t>
+    <t>Cô Thư (Ra đề); Cô Na (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Tú (Ra đề); Cô Như (Ra đề)</t>
+  </si>
+  <si>
+    <t>Cô Quí (Ra đề); Cô Bình (Phản biện)</t>
   </si>
   <si>
     <t>NGHIA</t>
@@ -426,40 +408,37 @@
     <t>Thầy Nghĩa</t>
   </si>
   <si>
-    <t>Cô Hiền (Ra đề); Cô Lài (Ra đề); Thầy Phúc (Phản biện); Cô Hiền (Phản biện)</t>
-  </si>
-  <si>
-    <t>Thầy Lộc (Ra đề); Cô Thư (Ra đề); Cô Na (Phản biện); Cô Lài (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Bình (Ra đề); Thầy Phúc (Ra đề); Cô Quí (Phản biện); Thầy Lộc (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Hiền (Ra đề); Cô Tú (Ra đề); Cô Như (Phản biện); Cô Tú (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Lài (Ra đề); Cô Bình (Ra đề); Cô Thư (Phản biện); Cô Lan (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Lan (Ra đề); Cô Quí (Ra đề); Cô Lài (Phản biện); Cô Bình (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Tú (Ra đề); Cô Như (Ra đề); Thầy Lộc (Phản biện); Cô Như (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Na (Ra đề); Cô Thư (Ra đề); Cô Hiền (Phản biện); Cô Thư (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Lan (Ra đề); Cô Lài (Ra đề); Cô Quí (Phản biện); Thầy Phúc (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Na (Ra đề); Cô Như (Ra đề); Cô Tú (Phản biện); Cô Quí (Phản biện)</t>
-  </si>
-  <si>
-    <t>Thầy Lộc (Ra đề); Cô Quí (Ra đề); Cô Bình (Phản biện); Cô Na (Phản biện)</t>
-  </si>
-  <si>
-    <t>Thầy Phúc (Ra đề); Cô Hiền (Ra đề); Cô Lan (Phản biện); Cô Quí (Phản biện)</t>
+    <t>Cô Hiền (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Lài (Phản biện)</t>
+  </si>
+  <si>
+    <t>Thầy Lộc (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Tú (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Lan (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Bình (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Như (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Thư (Phản biện)</t>
+  </si>
+  <si>
+    <t>Thầy Phúc (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Quí (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Na (Phản biện)</t>
   </si>
   <si>
     <t>PHUC</t>
@@ -468,16 +447,13 @@
     <t>Thầy Phúc</t>
   </si>
   <si>
-    <t>Cô Hiền (Ra đề); Cô Lài (Ra đề); Thầy Nghĩa (Ra đề); Cô Hiền (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Bình (Ra đề); Cô Quí (Phản biện); Thầy Nghĩa (Ra đề); Thầy Lộc (Phản biện)</t>
-  </si>
-  <si>
-    <t>Cô Lan (Ra đề); Cô Lài (Ra đề); Cô Quí (Phản biện); Thầy Nghĩa (Ra đề)</t>
-  </si>
-  <si>
-    <t>Cô Hiền (Ra đề); Cô Lan (Phản biện); Thầy Nghĩa (Ra đề); Cô Quí (Phản biện)</t>
+    <t>Cô Hiền (Ra đề); Cô Lài (Ra đề)</t>
+  </si>
+  <si>
+    <t>Cô Bình (Ra đề); Cô Quí (Phản biện)</t>
+  </si>
+  <si>
+    <t>Cô Hiền (Ra đề); Cô Lan (Phản biện)</t>
   </si>
   <si>
     <t>Số đề ra</t>
@@ -513,10 +489,13 @@
     <t>Đóng góp điểm</t>
   </si>
   <si>
+    <t>Cận dưới (đơn vị)</t>
+  </si>
+  <si>
     <t>H3</t>
   </si>
   <si>
-    <t>H3 - Đa dạng phân hiệu trong ban thi</t>
+    <t>H3 - Đa dạng phân hiệu</t>
   </si>
   <si>
     <t>Bật</t>
@@ -525,73 +504,73 @@
     <t>H4</t>
   </si>
   <si>
-    <t>H4 - Giới hạn số nhiệm vụ trong mỗi kỳ thi</t>
+    <t>H4 - Giới hạn nhiệm vụ trong mỗi kỳ thi</t>
   </si>
   <si>
     <t>H7</t>
   </si>
   <si>
-    <t>H7 - Cân bằng định mức công việc</t>
+    <t>H7 - Khung chỉ tiêu khối lượng</t>
   </si>
   <si>
     <t>S1</t>
   </si>
   <si>
-    <t>S1 - Phân bổ số lượt phản biện</t>
+    <t>S1 - Tần suất phản biện</t>
   </si>
   <si>
     <t>S2</t>
   </si>
   <si>
-    <t>S2 - Cân bằng vai trò ra đề / phản biện</t>
+    <t>S2 - Cân bằng tỷ lệ vai trò</t>
   </si>
   <si>
     <t>S3</t>
   </si>
   <si>
-    <t>S3 - Tránh liên tiếp 2 kỳ làm cùng vai trò</t>
+    <t>S3 - Phản biện độc lập phân hiệu</t>
   </si>
   <si>
     <t>S4</t>
   </si>
   <si>
-    <t>S4 - Tránh liên tiếp 2 kỳ làm cùng khối</t>
+    <t>S4 - Đa dạng cặp ra đề</t>
   </si>
   <si>
     <t>S5</t>
   </si>
   <si>
-    <t>S5 - Tránh cặp đôi lặp lại</t>
+    <t>S5 - Tránh phản biện chéo lặp lại</t>
   </si>
   <si>
     <t>S6</t>
   </si>
   <si>
-    <t>S6 - Tránh ban thi toàn giáo viên dạy khối đó</t>
+    <t>S6 - Giãn cách kỳ thi liên tiếp</t>
   </si>
   <si>
     <t>S7</t>
   </si>
   <si>
-    <t>S7 - Phân bổ đều giữa các khối</t>
+    <t>S7 - Luân chuyển khối lớp</t>
   </si>
   <si>
     <t>S8</t>
   </si>
   <si>
-    <t>S8 - Phân hiệu chính cho môn học</t>
+    <t>S8 - Cân bằng tải trọng thực tế</t>
   </si>
   <si>
     <t>S9</t>
   </si>
   <si>
-    <t>S9 - Hạn chế dồn nhiều nhiệm vụ trong một kỳ thi</t>
+    <t>S9 - Giảm dồn việc trong kỳ thi</t>
   </si>
   <si>
     <t>S10</t>
   </si>
   <si>
-    <t>S10 - Phản biện đủ các môn phụ trách</t>
+    <t>S10 - Phủ đủ môn phản biện</t>
   </si>
 </sst>
 </file>
@@ -2344,7 +2323,7 @@
         <v>72</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -2448,7 +2427,7 @@
         <v>72</v>
       </c>
       <c r="H11" s="19" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -2474,7 +2453,7 @@
         <v>68</v>
       </c>
       <c r="H12" s="19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -2500,7 +2479,7 @@
         <v>68</v>
       </c>
       <c r="H13" s="19" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -2526,18 +2505,18 @@
         <v>72</v>
       </c>
       <c r="H14" s="19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B15" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="C15" s="19" t="s">
         <v>89</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>90</v>
       </c>
       <c r="D15" s="17" t="s">
         <v>67</v>
@@ -2552,18 +2531,18 @@
         <v>68</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="C16" s="19" t="s">
         <v>89</v>
-      </c>
-      <c r="C16" s="19" t="s">
-        <v>90</v>
       </c>
       <c r="D16" s="17" t="s">
         <v>71</v>
@@ -2578,18 +2557,18 @@
         <v>72</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B17" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="C17" s="19" t="s">
         <v>89</v>
-      </c>
-      <c r="C17" s="19" t="s">
-        <v>90</v>
       </c>
       <c r="D17" s="17" t="s">
         <v>67</v>
@@ -2604,18 +2583,18 @@
         <v>68</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B18" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="C18" s="19" t="s">
         <v>89</v>
-      </c>
-      <c r="C18" s="19" t="s">
-        <v>90</v>
       </c>
       <c r="D18" s="17" t="s">
         <v>67</v>
@@ -2630,18 +2609,18 @@
         <v>72</v>
       </c>
       <c r="H18" s="19" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B19" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="C19" s="19" t="s">
         <v>89</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>90</v>
       </c>
       <c r="D19" s="17" t="s">
         <v>67</v>
@@ -2656,18 +2635,18 @@
         <v>68</v>
       </c>
       <c r="H19" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D20" s="17" t="s">
         <v>67</v>
@@ -2682,18 +2661,18 @@
         <v>72</v>
       </c>
       <c r="H20" s="19" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D21" s="17" t="s">
         <v>67</v>
@@ -2708,18 +2687,18 @@
         <v>68</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D22" s="17" t="s">
         <v>67</v>
@@ -2734,18 +2713,18 @@
         <v>68</v>
       </c>
       <c r="H22" s="19" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D23" s="17" t="s">
         <v>71</v>
@@ -2760,18 +2739,18 @@
         <v>72</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>101</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="17" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D24" s="17" t="s">
         <v>67</v>
@@ -2786,18 +2765,18 @@
         <v>72</v>
       </c>
       <c r="H24" s="19" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="17" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D25" s="17" t="s">
         <v>67</v>
@@ -2812,18 +2791,18 @@
         <v>68</v>
       </c>
       <c r="H25" s="19" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="17" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D26" s="17" t="s">
         <v>71</v>
@@ -2838,18 +2817,18 @@
         <v>72</v>
       </c>
       <c r="H26" s="19" t="s">
-        <v>105</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="17" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D27" s="17" t="s">
         <v>67</v>
@@ -2864,18 +2843,18 @@
         <v>68</v>
       </c>
       <c r="H27" s="19" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="17" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D28" s="17" t="s">
         <v>67</v>
@@ -2890,18 +2869,18 @@
         <v>72</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="17" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D29" s="17" t="s">
         <v>67</v>
@@ -2916,18 +2895,18 @@
         <v>68</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="17" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D30" s="17" t="s">
         <v>67</v>
@@ -2942,18 +2921,18 @@
         <v>72</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="17" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D31" s="17" t="s">
         <v>71</v>
@@ -2968,18 +2947,18 @@
         <v>72</v>
       </c>
       <c r="H31" s="19" t="s">
-        <v>113</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="17" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D32" s="17" t="s">
         <v>67</v>
@@ -2994,18 +2973,18 @@
         <v>68</v>
       </c>
       <c r="H32" s="19" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33" s="17" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D33" s="17" t="s">
         <v>71</v>
@@ -3020,15 +2999,15 @@
         <v>72</v>
       </c>
       <c r="H33" s="19" t="s">
-        <v>115</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" s="17" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C34" s="19" t="s">
         <v>77</v>
@@ -3046,15 +3025,15 @@
         <v>68</v>
       </c>
       <c r="H34" s="19" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="17" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C35" s="19" t="s">
         <v>77</v>
@@ -3072,15 +3051,15 @@
         <v>72</v>
       </c>
       <c r="H35" s="19" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="36" spans="1:8">
       <c r="A36" s="17" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C36" s="19" t="s">
         <v>77</v>
@@ -3098,15 +3077,15 @@
         <v>68</v>
       </c>
       <c r="H36" s="19" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="37" spans="1:8">
       <c r="A37" s="17" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C37" s="19" t="s">
         <v>77</v>
@@ -3124,15 +3103,15 @@
         <v>72</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>120</v>
+        <v>73</v>
       </c>
     </row>
     <row r="38" spans="1:8">
       <c r="A38" s="17" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C38" s="19" t="s">
         <v>77</v>
@@ -3150,15 +3129,15 @@
         <v>68</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="17" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C39" s="19" t="s">
         <v>77</v>
@@ -3176,15 +3155,15 @@
         <v>72</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>123</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" spans="1:8">
       <c r="A40" s="17" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C40" s="19" t="s">
         <v>77</v>
@@ -3202,15 +3181,15 @@
         <v>68</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="41" spans="1:8">
       <c r="A41" s="17" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C41" s="19" t="s">
         <v>77</v>
@@ -3228,18 +3207,18 @@
         <v>72</v>
       </c>
       <c r="H41" s="19" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
     <row r="42" spans="1:8">
       <c r="A42" s="17" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="C42" s="19" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D42" s="17" t="s">
         <v>67</v>
@@ -3254,18 +3233,18 @@
         <v>68</v>
       </c>
       <c r="H42" s="19" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="43" spans="1:8">
       <c r="A43" s="17" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="C43" s="19" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D43" s="17" t="s">
         <v>71</v>
@@ -3280,18 +3259,18 @@
         <v>72</v>
       </c>
       <c r="H43" s="19" t="s">
-        <v>129</v>
+        <v>73</v>
       </c>
     </row>
     <row r="44" spans="1:8">
       <c r="A44" s="17" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="C44" s="19" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D44" s="17" t="s">
         <v>67</v>
@@ -3306,18 +3285,18 @@
         <v>72</v>
       </c>
       <c r="H44" s="19" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="45" spans="1:8">
       <c r="A45" s="17" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="C45" s="19" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D45" s="17" t="s">
         <v>67</v>
@@ -3332,15 +3311,15 @@
         <v>68</v>
       </c>
       <c r="H45" s="19" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="46" spans="1:8">
       <c r="A46" s="17" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C46" s="19" t="s">
         <v>77</v>
@@ -3358,15 +3337,15 @@
         <v>68</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="47" spans="1:8">
       <c r="A47" s="17" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B47" s="19" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C47" s="19" t="s">
         <v>77</v>
@@ -3384,15 +3363,15 @@
         <v>68</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
     </row>
     <row r="48" spans="1:8">
       <c r="A48" s="17" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B48" s="19" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C48" s="19" t="s">
         <v>77</v>
@@ -3410,15 +3389,15 @@
         <v>68</v>
       </c>
       <c r="H48" s="19" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
     </row>
     <row r="49" spans="1:8">
       <c r="A49" s="17" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C49" s="19" t="s">
         <v>77</v>
@@ -3436,15 +3415,15 @@
         <v>68</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
     </row>
     <row r="50" spans="1:8">
       <c r="A50" s="17" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B50" s="19" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C50" s="19" t="s">
         <v>77</v>
@@ -3462,15 +3441,15 @@
         <v>68</v>
       </c>
       <c r="H50" s="19" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
     </row>
     <row r="51" spans="1:8">
       <c r="A51" s="17" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B51" s="19" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C51" s="19" t="s">
         <v>77</v>
@@ -3488,15 +3467,15 @@
         <v>68</v>
       </c>
       <c r="H51" s="19" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
     </row>
     <row r="52" spans="1:8">
       <c r="A52" s="17" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B52" s="19" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C52" s="19" t="s">
         <v>77</v>
@@ -3514,15 +3493,15 @@
         <v>68</v>
       </c>
       <c r="H52" s="19" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="53" spans="1:8">
       <c r="A53" s="17" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B53" s="19" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C53" s="19" t="s">
         <v>77</v>
@@ -3540,15 +3519,15 @@
         <v>68</v>
       </c>
       <c r="H53" s="19" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
     </row>
     <row r="54" spans="1:8">
       <c r="A54" s="17" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B54" s="19" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C54" s="19" t="s">
         <v>77</v>
@@ -3566,15 +3545,15 @@
         <v>68</v>
       </c>
       <c r="H54" s="19" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
     </row>
     <row r="55" spans="1:8">
       <c r="A55" s="17" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B55" s="19" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C55" s="19" t="s">
         <v>77</v>
@@ -3592,15 +3571,15 @@
         <v>68</v>
       </c>
       <c r="H55" s="19" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="56" spans="1:8">
       <c r="A56" s="17" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B56" s="19" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C56" s="19" t="s">
         <v>77</v>
@@ -3618,15 +3597,15 @@
         <v>68</v>
       </c>
       <c r="H56" s="19" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
     </row>
     <row r="57" spans="1:8">
       <c r="A57" s="17" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B57" s="19" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C57" s="19" t="s">
         <v>77</v>
@@ -3644,15 +3623,15 @@
         <v>68</v>
       </c>
       <c r="H57" s="19" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
     </row>
     <row r="58" spans="1:8">
       <c r="A58" s="17" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="B58" s="19" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C58" s="19" t="s">
         <v>66</v>
@@ -3670,15 +3649,15 @@
         <v>72</v>
       </c>
       <c r="H58" s="19" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
     </row>
     <row r="59" spans="1:8">
       <c r="A59" s="17" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="B59" s="19" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C59" s="19" t="s">
         <v>66</v>
@@ -3696,15 +3675,15 @@
         <v>68</v>
       </c>
       <c r="H59" s="19" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
     </row>
     <row r="60" spans="1:8">
       <c r="A60" s="17" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="B60" s="19" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C60" s="19" t="s">
         <v>66</v>
@@ -3722,15 +3701,15 @@
         <v>72</v>
       </c>
       <c r="H60" s="19" t="s">
-        <v>150</v>
+        <v>73</v>
       </c>
     </row>
     <row r="61" spans="1:8">
       <c r="A61" s="17" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="B61" s="19" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C61" s="19" t="s">
         <v>66</v>
@@ -3748,7 +3727,7 @@
         <v>68</v>
       </c>
       <c r="H61" s="19" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -3780,19 +3759,19 @@
         <v>60</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -3823,13 +3802,13 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B3" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="C3" s="19" t="s">
         <v>89</v>
-      </c>
-      <c r="C3" s="19" t="s">
-        <v>90</v>
       </c>
       <c r="D3" s="17">
         <v>3</v>
@@ -3849,10 +3828,10 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="17" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C4" s="19" t="s">
         <v>66</v>
@@ -3875,13 +3854,13 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="17" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D5" s="17">
         <v>2</v>
@@ -3901,10 +3880,10 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="17" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C6" s="19" t="s">
         <v>77</v>
@@ -3927,13 +3906,13 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D7" s="17">
         <v>2</v>
@@ -3979,13 +3958,13 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="17" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D9" s="17">
         <v>2</v>
@@ -4005,10 +3984,10 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="17" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C10" s="19" t="s">
         <v>77</v>
@@ -4031,13 +4010,13 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="17" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D11" s="17">
         <v>2</v>
@@ -4083,10 +4062,10 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="17" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C13" s="19" t="s">
         <v>77</v>
@@ -4114,44 +4093,48 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
     <col min="2" max="2" width="35.7109375" customWidth="1"/>
     <col min="3" max="4" width="14.7109375" customWidth="1"/>
     <col min="5" max="6" width="18.7109375" customWidth="1"/>
+    <col min="7" max="7" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="F1" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="G1" s="16" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="B2" s="19" t="s">
         <v>157</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C2" s="17" t="s">
         <v>158</v>
-      </c>
-      <c r="C1" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>160</v>
-      </c>
-      <c r="E1" s="16" t="s">
-        <v>161</v>
-      </c>
-      <c r="F1" s="16" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="17" t="s">
-        <v>163</v>
-      </c>
-      <c r="B2" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="C2" s="17" t="s">
-        <v>165</v>
       </c>
       <c r="D2" s="17">
         <v>100</v>
@@ -4162,16 +4145,19 @@
       <c r="F2" s="17">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="G2" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" s="17" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D3" s="17">
         <v>100</v>
@@ -4182,16 +4168,19 @@
       <c r="F3" s="17">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
+      <c r="G3" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4" s="17" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D4" s="17">
         <v>100</v>
@@ -4202,16 +4191,19 @@
       <c r="F4" s="17">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="G4" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" s="17" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D5" s="17">
         <v>10</v>
@@ -4222,16 +4214,19 @@
       <c r="F5" s="17">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="G5" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" s="17" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D6" s="17">
         <v>3</v>
@@ -4242,16 +4237,19 @@
       <c r="F6" s="17">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="G6" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7" s="17" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D7" s="17">
         <v>4</v>
@@ -4262,16 +4260,19 @@
       <c r="F7" s="17">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="G7" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" s="17" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D8" s="17">
         <v>6</v>
@@ -4282,16 +4283,19 @@
       <c r="F8" s="17">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="G8" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
       <c r="A9" s="17" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D9" s="17">
         <v>6</v>
@@ -4302,16 +4306,19 @@
       <c r="F9" s="17">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:6">
+      <c r="G9" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" s="17" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D10" s="17">
         <v>2</v>
@@ -4322,16 +4329,19 @@
       <c r="F10" s="17">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:6">
+      <c r="G10" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
       <c r="A11" s="17" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D11" s="17">
         <v>1</v>
@@ -4342,16 +4352,19 @@
       <c r="F11" s="17">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:6">
+      <c r="G11" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
       <c r="A12" s="17" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D12" s="17">
         <v>8</v>
@@ -4362,16 +4375,19 @@
       <c r="F12" s="17">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:6">
+      <c r="G12" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
       <c r="A13" s="17" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D13" s="17">
         <v>5</v>
@@ -4382,16 +4398,19 @@
       <c r="F13" s="17">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:6">
+      <c r="G13" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
       <c r="A14" s="17" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D14" s="17">
         <v>4</v>
@@ -4400,6 +4419,9 @@
         <v>0</v>
       </c>
       <c r="F14" s="17">
+        <v>0</v>
+      </c>
+      <c r="G14" s="17">
         <v>0</v>
       </c>
     </row>

</xml_diff>